<commit_message>
Updated the report: review figures, diagnostics, financial appendix
</commit_message>
<xml_diff>
--- a/python/results/results.xlsx
+++ b/python/results/results.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Monthly profit ($m)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Parameters" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly profit ($m)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financial model inputs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1652,6 +1653,644 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:N13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>scheme</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>energy_sold_gwh</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>capacity_factor</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>buy_p10</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>buy_mean</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>buy_p50</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>buy_p90</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>sell_p10</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>sell_mean</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>sell_p50</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>sell_p90</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>margin_per_mwh_sold</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>gross_profit_bn</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>S1 perfect foresight</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>5146.6</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.2671</v>
+      </c>
+      <c r="E2" t="n">
+        <v>9.449999999999999</v>
+      </c>
+      <c r="F2" t="n">
+        <v>101.39</v>
+      </c>
+      <c r="G2" t="n">
+        <v>82.66</v>
+      </c>
+      <c r="H2" t="n">
+        <v>247.4</v>
+      </c>
+      <c r="I2" t="n">
+        <v>119.37</v>
+      </c>
+      <c r="J2" t="n">
+        <v>307.74</v>
+      </c>
+      <c r="K2" t="n">
+        <v>240.68</v>
+      </c>
+      <c r="L2" t="n">
+        <v>508.32</v>
+      </c>
+      <c r="M2" t="n">
+        <v>172.07</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.886</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>S2 rule of thumb</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1547.7</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.0803</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-37.93</v>
+      </c>
+      <c r="F3" t="n">
+        <v>22.54</v>
+      </c>
+      <c r="G3" t="n">
+        <v>30.54</v>
+      </c>
+      <c r="H3" t="n">
+        <v>64.93000000000001</v>
+      </c>
+      <c r="I3" t="n">
+        <v>138.32</v>
+      </c>
+      <c r="J3" t="n">
+        <v>206.67</v>
+      </c>
+      <c r="K3" t="n">
+        <v>173.01</v>
+      </c>
+      <c r="L3" t="n">
+        <v>298.72</v>
+      </c>
+      <c r="M3" t="n">
+        <v>173.39</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.268</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>S3 forecaster</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>3410</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.1769</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-7.34</v>
+      </c>
+      <c r="F4" t="n">
+        <v>64.28</v>
+      </c>
+      <c r="G4" t="n">
+        <v>69.78</v>
+      </c>
+      <c r="H4" t="n">
+        <v>126.89</v>
+      </c>
+      <c r="I4" t="n">
+        <v>118.2</v>
+      </c>
+      <c r="J4" t="n">
+        <v>224.5</v>
+      </c>
+      <c r="K4" t="n">
+        <v>190.32</v>
+      </c>
+      <c r="L4" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="M4" t="n">
+        <v>137.02</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.467</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>S1 perfect foresight</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>5745</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.2981</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-22.14</v>
+      </c>
+      <c r="F5" t="n">
+        <v>38.84</v>
+      </c>
+      <c r="G5" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="H5" t="n">
+        <v>80.51000000000001</v>
+      </c>
+      <c r="I5" t="n">
+        <v>92.25</v>
+      </c>
+      <c r="J5" t="n">
+        <v>178.8</v>
+      </c>
+      <c r="K5" t="n">
+        <v>132.61</v>
+      </c>
+      <c r="L5" t="n">
+        <v>265.48</v>
+      </c>
+      <c r="M5" t="n">
+        <v>124.36</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.714</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>S2 rule of thumb</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2375.1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.1232</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-2.97</v>
+      </c>
+      <c r="F6" t="n">
+        <v>38.39</v>
+      </c>
+      <c r="G6" t="n">
+        <v>49.05</v>
+      </c>
+      <c r="H6" t="n">
+        <v>65.29000000000001</v>
+      </c>
+      <c r="I6" t="n">
+        <v>137.59</v>
+      </c>
+      <c r="J6" t="n">
+        <v>238.1</v>
+      </c>
+      <c r="K6" t="n">
+        <v>170.6</v>
+      </c>
+      <c r="L6" t="n">
+        <v>297.43</v>
+      </c>
+      <c r="M6" t="n">
+        <v>184.24</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.438</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>S3 forecaster</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>4838.9</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.2511</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-0.55</v>
+      </c>
+      <c r="F7" t="n">
+        <v>48.69</v>
+      </c>
+      <c r="G7" t="n">
+        <v>57.35</v>
+      </c>
+      <c r="H7" t="n">
+        <v>85.7</v>
+      </c>
+      <c r="I7" t="n">
+        <v>106.08</v>
+      </c>
+      <c r="J7" t="n">
+        <v>191.89</v>
+      </c>
+      <c r="K7" t="n">
+        <v>138.71</v>
+      </c>
+      <c r="L7" t="n">
+        <v>276.96</v>
+      </c>
+      <c r="M7" t="n">
+        <v>124.66</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.603</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>S1 perfect foresight</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>6528.7</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.3378</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-23.15</v>
+      </c>
+      <c r="F8" t="n">
+        <v>40.46</v>
+      </c>
+      <c r="G8" t="n">
+        <v>51.23</v>
+      </c>
+      <c r="H8" t="n">
+        <v>83.78</v>
+      </c>
+      <c r="I8" t="n">
+        <v>92.72</v>
+      </c>
+      <c r="J8" t="n">
+        <v>276.11</v>
+      </c>
+      <c r="K8" t="n">
+        <v>157.75</v>
+      </c>
+      <c r="L8" t="n">
+        <v>292.88</v>
+      </c>
+      <c r="M8" t="n">
+        <v>219.56</v>
+      </c>
+      <c r="N8" t="n">
+        <v>1.433</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>S2 rule of thumb</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>3017.1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.1561</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-30.48</v>
+      </c>
+      <c r="F9" t="n">
+        <v>31.78</v>
+      </c>
+      <c r="G9" t="n">
+        <v>45.7</v>
+      </c>
+      <c r="H9" t="n">
+        <v>64.18000000000001</v>
+      </c>
+      <c r="I9" t="n">
+        <v>139.81</v>
+      </c>
+      <c r="J9" t="n">
+        <v>382.15</v>
+      </c>
+      <c r="K9" t="n">
+        <v>185.15</v>
+      </c>
+      <c r="L9" t="n">
+        <v>299.66</v>
+      </c>
+      <c r="M9" t="n">
+        <v>336.87</v>
+      </c>
+      <c r="N9" t="n">
+        <v>1.016</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>S3 forecaster</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>5516.5</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.2855</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-16.33</v>
+      </c>
+      <c r="F10" t="n">
+        <v>44.98</v>
+      </c>
+      <c r="G10" t="n">
+        <v>54.06</v>
+      </c>
+      <c r="H10" t="n">
+        <v>85.45999999999999</v>
+      </c>
+      <c r="I10" t="n">
+        <v>105.54</v>
+      </c>
+      <c r="J10" t="n">
+        <v>301.23</v>
+      </c>
+      <c r="K10" t="n">
+        <v>164.37</v>
+      </c>
+      <c r="L10" t="n">
+        <v>294.26</v>
+      </c>
+      <c r="M10" t="n">
+        <v>238.82</v>
+      </c>
+      <c r="N10" t="n">
+        <v>1.317</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>S1 perfect foresight</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>6680.1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.3466</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-19.19</v>
+      </c>
+      <c r="F11" t="n">
+        <v>28.72</v>
+      </c>
+      <c r="G11" t="n">
+        <v>35.35</v>
+      </c>
+      <c r="H11" t="n">
+        <v>73.06999999999999</v>
+      </c>
+      <c r="I11" t="n">
+        <v>101.91</v>
+      </c>
+      <c r="J11" t="n">
+        <v>210.16</v>
+      </c>
+      <c r="K11" t="n">
+        <v>140.06</v>
+      </c>
+      <c r="L11" t="n">
+        <v>242.35</v>
+      </c>
+      <c r="M11" t="n">
+        <v>168.86</v>
+      </c>
+      <c r="N11" t="n">
+        <v>1.128</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>S2 rule of thumb</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>3587.2</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.1861</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-17.5</v>
+      </c>
+      <c r="F12" t="n">
+        <v>25.22</v>
+      </c>
+      <c r="G12" t="n">
+        <v>30.82</v>
+      </c>
+      <c r="H12" t="n">
+        <v>62.94</v>
+      </c>
+      <c r="I12" t="n">
+        <v>138.41</v>
+      </c>
+      <c r="J12" t="n">
+        <v>288.75</v>
+      </c>
+      <c r="K12" t="n">
+        <v>167.06</v>
+      </c>
+      <c r="L12" t="n">
+        <v>278.52</v>
+      </c>
+      <c r="M12" t="n">
+        <v>252</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.904</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>S3 forecaster</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>5932.3</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.3078</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-18.33</v>
+      </c>
+      <c r="F13" t="n">
+        <v>33.21</v>
+      </c>
+      <c r="G13" t="n">
+        <v>39.74</v>
+      </c>
+      <c r="H13" t="n">
+        <v>77.69</v>
+      </c>
+      <c r="I13" t="n">
+        <v>107.16</v>
+      </c>
+      <c r="J13" t="n">
+        <v>223.02</v>
+      </c>
+      <c r="K13" t="n">
+        <v>145.82</v>
+      </c>
+      <c r="L13" t="n">
+        <v>249.65</v>
+      </c>
+      <c r="M13" t="n">
+        <v>175.89</v>
+      </c>
+      <c r="N13" t="n">
+        <v>1.043</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>